<commit_message>
Improve article pages: white background, date line, hero image
- Update transformer to preserve date/author line and hero image
- Add white card background matching original Microsoft Blog layout
- Style date line in gray with positional CSS selectors
- Hero image renders edge-to-edge within the content card
- Re-import all 14 articles with updated transformer

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-ms-blog-article.report.xlsx
+++ b/tools/importer/reports/import-ms-blog-article.report.xlsx
@@ -73,7 +73,7 @@
     <t>ms-blog-article</t>
   </si>
   <si>
-    <t>2026-03-17T21:48:20.046Z</t>
+    <t>2026-03-17T22:30:56.983Z</t>
   </si>
   <si>
     <t>From idea to deployment: The complete lifecycle of AI on display at Ignite 2025 - The Official Microsoft Blog</t>
@@ -88,7 +88,7 @@
     <t>blog/2026/01/05/microsoft-announces-acquisition-of-osmos-to-accelerate-autonomous-data-engineering-in-fabric</t>
   </si>
   <si>
-    <t>2026-03-17T21:48:14.757Z</t>
+    <t>2026-03-17T22:30:52.438Z</t>
   </si>
   <si>
     <t>Microsoft announces acquisition of Osmos to accelerate autonomous data engineering in Fabric - The Official Microsoft Blog</t>
@@ -103,7 +103,7 @@
     <t>blog/2026/01/13/announcing-open-to-work-how-to-get-ahead-in-the-age-of-ai</t>
   </si>
   <si>
-    <t>2026-03-17T21:48:10.879Z</t>
+    <t>2026-03-17T22:30:46.747Z</t>
   </si>
   <si>
     <t>Announcing Open to Work: How to Get Ahead in the Age of AI - The Official Microsoft Blog</t>
@@ -118,7 +118,7 @@
     <t>blog/2026/01/26/maia-200-the-ai-accelerator-built-for-inference</t>
   </si>
   <si>
-    <t>2026-03-17T21:48:06.219Z</t>
+    <t>2026-03-17T22:30:40.843Z</t>
   </si>
   <si>
     <t>Maia 200: The AI accelerator built for inference - The Official Microsoft Blog</t>
@@ -133,7 +133,7 @@
     <t>blog/2026/01/27/how-microsoft-is-empowering-frontier-transformation-with-intelligence-trust</t>
   </si>
   <si>
-    <t>2026-03-17T21:48:02.037Z</t>
+    <t>2026-03-17T22:30:35.952Z</t>
   </si>
   <si>
     <t>How Microsoft is empowering Frontier Transformation with Intelligence + Trust - The Official Microsoft Blog</t>
@@ -148,7 +148,7 @@
     <t>blog/2026/02/04/updates-in-two-of-our-core-priorities</t>
   </si>
   <si>
-    <t>2026-03-17T21:47:57.703Z</t>
+    <t>2026-03-17T22:30:30.140Z</t>
   </si>
   <si>
     <t>Updates in two of our core priorities - The Official Microsoft Blog</t>
@@ -163,7 +163,7 @@
     <t>blog/2026/02/18/a-milestone-achievement-in-our-journey-to-carbon-negative</t>
   </si>
   <si>
-    <t>2026-03-17T21:47:53.546Z</t>
+    <t>2026-03-17T22:30:25.384Z</t>
   </si>
   <si>
     <t>A milestone achievement in our journey to carbon negative - The Official Microsoft Blog</t>
@@ -178,7 +178,7 @@
     <t>blog/2026/02/20/asha-sharma-named-evp-and-ceo-microsoft-gaming</t>
   </si>
   <si>
-    <t>2026-03-17T21:47:47.369Z</t>
+    <t>2026-03-17T22:30:20.658Z</t>
   </si>
   <si>
     <t>Asha Sharma named EVP and CEO, Microsoft Gaming - The Official Microsoft Blog</t>
@@ -193,7 +193,7 @@
     <t>blog/2026/02/24/microsoft-sovereign-cloud-adds-governance-productivity-and-support-for-large-ai-models-securely-running-even-when-completely-disconnected</t>
   </si>
   <si>
-    <t>2026-03-17T21:47:42.498Z</t>
+    <t>2026-03-17T22:30:16.270Z</t>
   </si>
   <si>
     <t>Microsoft Sovereign Cloud adds governance, productivity and support for large AI models securely running even when completely disconnected  - The Official Microsoft Blog</t>
@@ -208,7 +208,7 @@
     <t>blog/2026/02/27/microsoft-and-openai-joint-statement-on-continuing-partnership</t>
   </si>
   <si>
-    <t>2026-03-17T21:47:36.921Z</t>
+    <t>2026-03-17T22:30:10.676Z</t>
   </si>
   <si>
     <t>Microsoft and OpenAI joint statement on continuing partnership - The Official Microsoft Blog</t>
@@ -223,7 +223,7 @@
     <t>blog/2026/03/09/introducing-the-first-frontier-suite-built-on-intelligence-trust</t>
   </si>
   <si>
-    <t>2026-03-17T21:47:33.489Z</t>
+    <t>2026-03-17T22:30:05.479Z</t>
   </si>
   <si>
     <t>Introducing the First Frontier Suite built on Intelligence + Trust - The Official Microsoft Blog</t>
@@ -238,7 +238,7 @@
     <t>blog/2026/03/12/microsoft-announces-experiences-devices-leadership-changes</t>
   </si>
   <si>
-    <t>2026-03-17T21:47:29.455Z</t>
+    <t>2026-03-17T22:29:59.428Z</t>
   </si>
   <si>
     <t>Microsoft announces Experiences + Devices leadership changes - The Official Microsoft Blog</t>
@@ -253,7 +253,7 @@
     <t>blog/2026/03/16/microsoft-at-nvidia-gtc-new-solutions-for-microsoft-foundry-azure-ai-infrastructure-and-physical-ai</t>
   </si>
   <si>
-    <t>2026-03-17T21:47:25.354Z</t>
+    <t>2026-03-17T22:29:55.275Z</t>
   </si>
   <si>
     <t>Microsoft at NVIDIA GTC: New solutions for Microsoft Foundry, Azure AI infrastructure and Physical AI - The Official Microsoft Blog</t>
@@ -268,7 +268,7 @@
     <t>blog/2026/03/17/announcing-copilot-leadership-update</t>
   </si>
   <si>
-    <t>2026-03-17T21:47:21.164Z</t>
+    <t>2026-03-17T22:29:49.672Z</t>
   </si>
   <si>
     <t>Announcing Copilot leadership update - The Official Microsoft Blog</t>

</xml_diff>